<commit_message>
Fix script. Change card: Mine card is removed and Caltrop card is added. Caltrop -> Territory. Whenever a card in its territory moved to another room in its territory, decrease the rank of that card by 1. Rule change: the player can stall for free once every floor reset.
</commit_message>
<xml_diff>
--- a/sheet/TerritoryCardData.xlsx
+++ b/sheet/TerritoryCardData.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Workspace\nanDeck\DungeonCrawlDeckMaster\sheet\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9FAD2330-F8BE-4C41-A84B-D851E4527FD3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1D2100DA-FDEB-4C09-8DAD-27326196654D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="6060" yWindow="2625" windowWidth="21600" windowHeight="11295" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="19" uniqueCount="19">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="21" uniqueCount="21">
   <si>
     <t>cardName</t>
     <phoneticPr fontId="1" type="noConversion"/>
@@ -98,6 +98,14 @@
   </si>
   <si>
     <t>领域内怪物牌死亡时：每张死亡的怪物牌使玩家额外获得1金币。</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>蒺藜</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>领域内的怪物牌移动到领域内的房间时：那张牌点数减1。</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
@@ -150,13 +158,12 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="常规" xfId="0" builtinId="0"/>
@@ -438,7 +445,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:E6"/>
+  <dimension ref="A1:E7"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.2">
@@ -501,7 +508,7 @@
       <c r="A5" t="s">
         <v>14</v>
       </c>
-      <c r="B5" s="3">
+      <c r="B5">
         <v>2</v>
       </c>
       <c r="C5" t="s">
@@ -523,6 +530,17 @@
       </c>
       <c r="C6" t="s">
         <v>18</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A7" t="s">
+        <v>19</v>
+      </c>
+      <c r="B7">
+        <v>2</v>
+      </c>
+      <c r="C7" t="s">
+        <v>20</v>
       </c>
     </row>
   </sheetData>

</xml_diff>